<commit_message>
feat: configure five sweep cards for player deck
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/SkillCardRule.xlsx
+++ b/Design/Excel/ET/Datas/Game/SkillCardRule.xlsx
@@ -574,10 +574,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
feat: add init mp to skill card rule
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/SkillCardRule.xlsx
+++ b/Design/Excel/ET/Datas/Game/SkillCardRule.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
           <t>PassiveTriggerIntervalSeconds</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>InitMp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -494,6 +499,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +536,11 @@
           <t>c</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -561,6 +576,11 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>PassiveTriggerIntervalSeconds</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>InitMp</t>
         </is>
       </c>
     </row>
@@ -587,6 +607,9 @@
       </c>
       <c r="H5" t="n">
         <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>